<commit_message>
data(ACC): unify ACC coding to the database-wide 6-code set
- Sui_2015_unpub: author codes 3=timeout (RT>=1000 ms) -> -4 (213 cells), 4=no response -> NA (6 cells); merge.R gains the mapping, stopifnot row-count guards and na="NA"; codebook ACC row updated
- Lee_2026_BritJPsy E1a/E1b/E2: empty ACC fields -> literal NA (1,417 cells); clean.R writes with na="NA"
- library-wide ACC domain now {1, 0, NA, -2, -4}; 0 out-of-domain cells; byte format (no BOM, LF) preserved
</commit_message>
<xml_diff>
--- a/1_Data/Sui_2015_unpub/Codebook_Sui_2015_unpub_Exp1_Clean.xlsx
+++ b/1_Data/Sui_2015_unpub/Codebook_Sui_2015_unpub_Exp1_Clean.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t xml:space="preserve">Variable_name</t>
   </si>
@@ -168,6 +168,12 @@
   </si>
   <si>
     <t xml:space="preserve">1;0;3;4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accuracy: 1 (correct); 0 (incorrect); -4 (response after the 1000 ms deadline; author raw code 3); NA (no response; author raw code 4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 (correct); 0 (incorrect); -4 (response after the 1000 ms deadline); NA (no response)</t>
   </si>
 </sst>
 </file>
@@ -767,10 +773,10 @@
         <v>49</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>

</xml_diff>